<commit_message>
Reset frontend model history and update collection
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1116ED6-D4A1-46A9-B5F3-E98F6E02C182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AE4D11E-05C6-4261-A0EC-07285F06D5F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
+    <workbookView xWindow="-38520" yWindow="-1575" windowWidth="38640" windowHeight="21120" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7580" uniqueCount="669">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7595" uniqueCount="669">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -2180,7 +2180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2221,19 +2221,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2583,7 +2570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E1537"/>
+  <dimension ref="A1:E1540"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -28263,36 +28250,36 @@
       </c>
     </row>
     <row r="1532" spans="1:5">
-      <c r="A1532" s="16" t="s">
+      <c r="A1532" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B1532" s="17" t="s">
+      <c r="B1532" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C1532" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1532" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1532" s="18" t="s">
+      <c r="C1532" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1532" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1532" s="7" t="s">
         <v>640</v>
       </c>
     </row>
     <row r="1533" spans="1:5">
-      <c r="A1533" s="16" t="s">
+      <c r="A1533" s="5" t="s">
         <v>49</v>
       </c>
       <c r="B1533" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C1533" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1533" s="17" t="s">
+      <c r="C1533" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1533" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E1533" s="18" t="s">
+      <c r="E1533" s="7" t="s">
         <v>640</v>
       </c>
     </row>
@@ -28300,7 +28287,7 @@
       <c r="A1534" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="B1534" s="17" t="s">
+      <c r="B1534" s="3" t="s">
         <v>58</v>
       </c>
       <c r="C1534" t="s">
@@ -28314,10 +28301,10 @@
       </c>
     </row>
     <row r="1535" spans="1:5" ht="15">
-      <c r="A1535" s="19" t="s">
+      <c r="A1535" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="B1535" s="17" t="s">
+      <c r="B1535" s="3" t="s">
         <v>58</v>
       </c>
       <c r="C1535" t="s">
@@ -28331,10 +28318,10 @@
       </c>
     </row>
     <row r="1536" spans="1:5" ht="15">
-      <c r="A1536" s="19" t="s">
+      <c r="A1536" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="B1536" s="20" t="s">
+      <c r="B1536" s="2" t="s">
         <v>76</v>
       </c>
       <c r="C1536" t="s">
@@ -28348,10 +28335,10 @@
       </c>
     </row>
     <row r="1537" spans="1:5" ht="15">
-      <c r="A1537" s="19" t="s">
+      <c r="A1537" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="B1537" s="20" t="s">
+      <c r="B1537" s="2" t="s">
         <v>76</v>
       </c>
       <c r="C1537" t="s">
@@ -28362,6 +28349,57 @@
       </c>
       <c r="E1537" s="2" t="s">
         <v>658</v>
+      </c>
+    </row>
+    <row r="1538" spans="1:5" ht="15">
+      <c r="A1538" s="1" t="s">
+        <v>643</v>
+      </c>
+      <c r="B1538" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1538" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1538" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1538" s="15" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="1539" spans="1:5" ht="15">
+      <c r="A1539" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B1539" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1539" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1539" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1539" s="15" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="1540" spans="1:5" ht="15">
+      <c r="A1540" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B1540" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1540" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1540" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1540" s="15" t="s">
+        <v>648</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update investment display and collection
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{090635A8-1DB6-45B9-8C8C-643B43AEEA53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA838C9-0097-4AA5-9D52-361D3BDF4A5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-1575" windowWidth="38640" windowHeight="21120" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
+    <workbookView xWindow="-38535" yWindow="-1590" windowWidth="38670" windowHeight="21150" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7690" uniqueCount="671">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7700" uniqueCount="671">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -2576,7 +2577,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E1562"/>
+  <dimension ref="A1:E1564"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -28731,6 +28732,40 @@
         <v>640</v>
       </c>
     </row>
+    <row r="1563" spans="1:5" ht="15">
+      <c r="A1563" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1563" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1563" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1563" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1563" s="7" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1564" spans="1:5" ht="15">
+      <c r="A1564" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1564" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1564" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1564" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1564" s="7" t="s">
+        <v>365</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}"/>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
Update summary tables and collection
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C63FABCA-4B0D-474C-8917-FD25275C213F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{063A00DA-4FC5-4B62-8734-CB0447116231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8360" uniqueCount="694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8375" uniqueCount="695">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -2121,6 +2121,9 @@
   </si>
   <si>
     <t>Throne of Bone</t>
+  </si>
+  <si>
+    <t>Greed</t>
   </si>
 </sst>
 </file>
@@ -2255,7 +2258,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2296,9 +2299,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2648,7 +2648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E1753"/>
+  <dimension ref="A1:E1756"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -30973,7 +30973,7 @@
       <c r="D1746" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1746" s="16" t="s">
+      <c r="E1746" s="8" t="s">
         <v>676</v>
       </c>
     </row>
@@ -30990,7 +30990,7 @@
       <c r="D1747" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1747" s="16" t="s">
+      <c r="E1747" s="8" t="s">
         <v>676</v>
       </c>
     </row>
@@ -31007,7 +31007,7 @@
       <c r="D1748" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1748" s="16" t="s">
+      <c r="E1748" s="8" t="s">
         <v>676</v>
       </c>
     </row>
@@ -31024,7 +31024,7 @@
       <c r="D1749" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1749" s="16" t="s">
+      <c r="E1749" s="8" t="s">
         <v>676</v>
       </c>
     </row>
@@ -31041,7 +31041,7 @@
       <c r="D1750" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1750" s="16" t="s">
+      <c r="E1750" s="8" t="s">
         <v>676</v>
       </c>
     </row>
@@ -31058,7 +31058,7 @@
       <c r="D1751" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E1751" s="16" t="s">
+      <c r="E1751" s="8" t="s">
         <v>676</v>
       </c>
     </row>
@@ -31075,7 +31075,7 @@
       <c r="D1752" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1752" s="16" t="s">
+      <c r="E1752" s="8" t="s">
         <v>676</v>
       </c>
     </row>
@@ -31092,8 +31092,59 @@
       <c r="D1753" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1753" s="16" t="s">
+      <c r="E1753" s="8" t="s">
         <v>676</v>
+      </c>
+    </row>
+    <row r="1754" spans="1:5" ht="15">
+      <c r="A1754" t="s">
+        <v>163</v>
+      </c>
+      <c r="B1754" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1754" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1754" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1754" s="2" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="1755" spans="1:5" ht="15">
+      <c r="A1755" s="1" t="s">
+        <v>694</v>
+      </c>
+      <c r="B1755" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1755" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1755" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1755" s="8" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="1756" spans="1:5" ht="15">
+      <c r="A1756" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B1756" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1756" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1756" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1756" s="2" t="s">
+        <v>648</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update MTG collection Excel
</commit_message>
<xml_diff>
--- a/uploads/collection.xlsx
+++ b/uploads/collection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sokom\Documents\mtg-portfolio2\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{063A00DA-4FC5-4B62-8734-CB0447116231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36344522-2ECD-4A3E-AABF-73433D81910A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0FB49C1A-78A4-4DA0-A11D-346B115E728B}"/>
   </bookViews>
@@ -19,6 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8375" uniqueCount="695">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8725" uniqueCount="706">
   <si>
     <t>Llanowar Elves</t>
   </si>
@@ -2124,6 +2125,39 @@
   </si>
   <si>
     <t>Greed</t>
+  </si>
+  <si>
+    <t>Stasis</t>
+  </si>
+  <si>
+    <t>Underground Sea</t>
+  </si>
+  <si>
+    <t>Phantom Monster</t>
+  </si>
+  <si>
+    <t>Orcish Oriflamme</t>
+  </si>
+  <si>
+    <t>Smoke</t>
+  </si>
+  <si>
+    <t>Roc of Kher Ridges</t>
+  </si>
+  <si>
+    <t>Earthbind </t>
+  </si>
+  <si>
+    <t>Wooden Sphere</t>
+  </si>
+  <si>
+    <t>Veteran Bodyguard</t>
+  </si>
+  <si>
+    <t>Rocket Launcher</t>
+  </si>
+  <si>
+    <t>Mountain (V.1) </t>
   </si>
 </sst>
 </file>
@@ -2258,7 +2292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2301,6 +2335,16 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2648,7 +2692,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCD6AFAC-F407-46DB-91C7-9730E2D3F96A}">
-  <dimension ref="A1:E1756"/>
+  <dimension ref="A1:E1830"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30.54296875" customWidth="1"/>
@@ -28206,74 +28250,6 @@
         <v>671</v>
       </c>
     </row>
-    <row r="1581" spans="1:5" ht="15">
-      <c r="A1581" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="B1581" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C1581" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1581" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1581" s="2" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="1582" spans="1:5" ht="15">
-      <c r="A1582" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="B1582" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C1582" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1582" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1582" s="2" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="1583" spans="1:5" ht="15">
-      <c r="A1583" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="B1583" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C1583" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1583" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1583" s="2" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="1584" spans="1:5" ht="15">
-      <c r="A1584" s="1" t="s">
-        <v>543</v>
-      </c>
-      <c r="B1584" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C1584" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1584" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E1584" s="2" t="s">
-        <v>671</v>
-      </c>
-    </row>
     <row r="1585" spans="1:5" ht="15">
       <c r="A1585" s="1" t="s">
         <v>472</v>
@@ -29944,11 +29920,11 @@
       <c r="A1686" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B1686" s="1" t="s">
-        <v>76</v>
+      <c r="B1686" s="3" t="s">
+        <v>28</v>
       </c>
       <c r="C1686" s="2" t="s">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="D1686" s="2" t="s">
         <v>6</v>
@@ -31145,6 +31121,1264 @@
       </c>
       <c r="E1756" s="2" t="s">
         <v>648</v>
+      </c>
+    </row>
+    <row r="1757" spans="1:5" ht="15">
+      <c r="A1757" s="1" t="s">
+        <v>695</v>
+      </c>
+      <c r="B1757" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1757" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1757" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1757" s="8" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1758" spans="1:5" ht="15">
+      <c r="A1758" s="1" t="s">
+        <v>696</v>
+      </c>
+      <c r="B1758" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1758" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1758" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1758" s="8" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="1759" spans="1:5" ht="15">
+      <c r="A1759" s="1" t="s">
+        <v>660</v>
+      </c>
+      <c r="B1759" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1759" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1759" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1759" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1760" spans="1:5" ht="15">
+      <c r="A1760" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="B1760" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1760" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1760" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1760" s="8" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="1761" spans="1:5" ht="15">
+      <c r="A1761" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="B1761" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1761" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1761" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1761" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1762" spans="1:5" ht="15">
+      <c r="A1762" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1762" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1762" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1762" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1762" s="8" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="1763" spans="1:5" ht="15">
+      <c r="A1763" s="1" t="s">
+        <v>678</v>
+      </c>
+      <c r="B1763" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1763" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1763" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1763" s="8" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1764" spans="1:5" ht="15">
+      <c r="A1764" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1764" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1764" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1764" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1764" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1765" spans="1:5" ht="15">
+      <c r="A1765" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="B1765" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1765" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1765" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1765" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1766" spans="1:5" ht="15">
+      <c r="A1766" s="1" t="s">
+        <v>699</v>
+      </c>
+      <c r="B1766" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1766" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1766" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1766" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1767" spans="1:5" ht="15">
+      <c r="A1767" s="1" t="s">
+        <v>700</v>
+      </c>
+      <c r="B1767" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1767" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1767" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1767" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1768" spans="1:5" ht="15">
+      <c r="A1768" s="1" t="s">
+        <v>701</v>
+      </c>
+      <c r="B1768" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1768" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1768" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1768" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1769" spans="1:5" ht="15">
+      <c r="A1769" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="B1769" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1769" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1769" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1769" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1770" spans="1:5" ht="15">
+      <c r="A1770" s="1" t="s">
+        <v>702</v>
+      </c>
+      <c r="B1770" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1770" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1770" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1770" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1771" spans="1:5" ht="15">
+      <c r="A1771" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B1771" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1771" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1771" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1771" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1772" spans="1:5" ht="15">
+      <c r="A1772" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B1772" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1772" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1772" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1772" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1773" spans="1:5" ht="15">
+      <c r="A1773" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B1773" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1773" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1773" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1773" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1774" spans="1:5" ht="15">
+      <c r="A1774" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B1774" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1774" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1774" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1774" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1775" spans="1:5" ht="15">
+      <c r="A1775" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B1775" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1775" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1775" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1775" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1776" spans="1:5" ht="15">
+      <c r="A1776" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B1776" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1776" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1776" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1776" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1777" spans="1:5" ht="15">
+      <c r="A1777" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B1777" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1777" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1777" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1777" s="2" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="1778" spans="1:5" ht="15">
+      <c r="A1778" s="1" t="s">
+        <v>703</v>
+      </c>
+      <c r="B1778" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1778" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1778" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1778" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1779" spans="1:5" ht="15">
+      <c r="A1779" s="1" t="s">
+        <v>704</v>
+      </c>
+      <c r="B1779" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1779" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1779" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1779" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1780" spans="1:5" ht="15">
+      <c r="A1780" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1780" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1780" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1780" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1780" s="18" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1781" spans="1:5" ht="15">
+      <c r="A1781" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="B1781" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1781" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1781" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1781" s="15" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="1782" spans="1:5" ht="15">
+      <c r="A1782" s="19" t="s">
+        <v>536</v>
+      </c>
+      <c r="B1782" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1782" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1782" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1782" s="18" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1783" spans="1:5">
+      <c r="A1783" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1783" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1783" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1783" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1783" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1784" spans="1:5" ht="15">
+      <c r="A1784" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1784" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1784" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1784" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1784" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1785" spans="1:5" ht="15">
+      <c r="A1785" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1785" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1785" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1785" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1785" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1786" spans="1:5" ht="15">
+      <c r="A1786" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1786" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1786" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1786" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1786" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1787" spans="1:5" ht="15">
+      <c r="A1787" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1787" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1787" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1787" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1787" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1788" spans="1:5" ht="15">
+      <c r="A1788" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1788" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1788" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1788" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1788" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1789" spans="1:5" ht="15">
+      <c r="A1789" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1789" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1789" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1789" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1789" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1790" spans="1:5" ht="15">
+      <c r="A1790" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1790" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1790" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1790" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1790" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1791" spans="1:5">
+      <c r="A1791" t="s">
+        <v>651</v>
+      </c>
+      <c r="B1791" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1791" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1791" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1791" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="1792" spans="1:5" ht="15">
+      <c r="A1792" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="B1792" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1792" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1792" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1792" s="8" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="1793" spans="1:5" ht="15">
+      <c r="A1793" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="B1793" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1793" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1793" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1793" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1794" spans="1:5" ht="15">
+      <c r="A1794" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="B1794" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1794" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1794" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1794" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1795" spans="1:5" ht="15">
+      <c r="A1795" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1795" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1795" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1795" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1795" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1796" spans="1:5" ht="15">
+      <c r="A1796" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1796" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1796" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1796" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1796" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1797" spans="1:5" ht="15">
+      <c r="A1797" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1797" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1797" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1797" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1797" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1798" spans="1:5" ht="15">
+      <c r="A1798" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1798" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1798" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1798" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1798" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1799" spans="1:5" ht="15">
+      <c r="A1799" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1799" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1799" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1799" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1799" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1800" spans="1:5" ht="15">
+      <c r="A1800" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1800" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1800" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1800" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1800" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1801" spans="1:5" ht="15">
+      <c r="A1801" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="B1801" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1801" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1801" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1801" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1802" spans="1:5" ht="15">
+      <c r="A1802" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="B1802" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1802" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1802" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1802" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1803" spans="1:5" ht="15">
+      <c r="A1803" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1803" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1803" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1803" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1803" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1804" spans="1:5" ht="15">
+      <c r="A1804" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1804" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1804" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1804" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1804" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1805" spans="1:5" ht="15">
+      <c r="A1805" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1805" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1805" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1805" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1805" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1806" spans="1:5" ht="15">
+      <c r="A1806" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1806" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1806" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1806" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1806" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1807" spans="1:5" ht="15">
+      <c r="A1807" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1807" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1807" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1807" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1807" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1808" spans="1:5" ht="15">
+      <c r="A1808" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1808" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1808" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1808" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1808" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1809" spans="1:5" ht="15">
+      <c r="A1809" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1809" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1809" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1809" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1809" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1810" spans="1:5" ht="15">
+      <c r="A1810" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1810" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1810" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1810" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1810" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1811" spans="1:5" ht="15">
+      <c r="A1811" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1811" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1811" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1811" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1811" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1812" spans="1:5" ht="15">
+      <c r="A1812" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1812" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1812" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1812" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1812" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1813" spans="1:5" ht="15">
+      <c r="A1813" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B1813" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1813" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1813" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1813" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1814" spans="1:5" ht="15">
+      <c r="A1814" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1814" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1814" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1814" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1814" s="2" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="1815" spans="1:5" ht="15">
+      <c r="A1815" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="B1815" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1815" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1815" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1815" s="2" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="1816" spans="1:5" ht="15">
+      <c r="A1816" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="B1816" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1816" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1816" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1816" s="2" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="1817" spans="1:5" ht="15">
+      <c r="A1817" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="B1817" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1817" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1817" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1817" s="2" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="1818" spans="1:5" ht="15">
+      <c r="A1818" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B1818" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1818" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1818" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1818" s="2" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="1819" spans="1:5" ht="15">
+      <c r="A1819" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B1819" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1819" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1819" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1819" s="2" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="1820" spans="1:5" ht="15">
+      <c r="A1820" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B1820" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1820" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1820" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1820" s="2" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="1821" spans="1:5" ht="15">
+      <c r="A1821" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B1821" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1821" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1821" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1821" s="2" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="1822" spans="1:5" ht="15">
+      <c r="A1822" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B1822" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1822" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1822" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1822" s="2" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="1823" spans="1:5" ht="15">
+      <c r="A1823" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B1823" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1823" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1823" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1823" s="2" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="1824" spans="1:5" ht="15">
+      <c r="A1824" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B1824" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1824" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1824" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1824" s="2" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="1825" spans="1:5" ht="15">
+      <c r="A1825" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B1825" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1825" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1825" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1825" s="2" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="1826" spans="1:5" ht="15">
+      <c r="A1826" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="B1826" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1826" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1826" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1826" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1827" spans="1:5" ht="15">
+      <c r="A1827" s="1" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1827" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1827" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1827" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1827" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1828" spans="1:5" ht="15">
+      <c r="A1828" s="1" t="s">
+        <v>705</v>
+      </c>
+      <c r="B1828" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1828" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1828" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1828" s="2" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="1829" spans="1:5" ht="15">
+      <c r="A1829" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B1829" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1829" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1829" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1829" s="2" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="1830" spans="1:5" ht="15">
+      <c r="A1830" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="B1830" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1830" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1830" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1830" s="2" t="s">
+        <v>680</v>
       </c>
     </row>
   </sheetData>

</xml_diff>